<commit_message>
Revision of Branding from USAID Tujenge Jamii to Tujenge Jamii
This upgrade works to comply to the new project branding
</commit_message>
<xml_diff>
--- a/web/hca.xlsx
+++ b/web/hca.xlsx
@@ -1,16 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\InternalSystem\web\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF5D5DD9-76B5-4919-A8E2-7E925E9C7029}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookPassword="CC71" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19320" windowHeight="7335" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="3" r:id="rId1"/>
@@ -26,7 +27,7 @@
     <definedName name="Test" localSheetId="0">#REF!</definedName>
     <definedName name="Test">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,6 +40,9 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -498,13 +502,13 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="yyyy/mmm"/>
   </numFmts>
-  <fonts count="48">
+  <fonts count="48" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3031,6 +3035,66 @@
     <xf numFmtId="0" fontId="40" fillId="17" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="38" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="17" fontId="14" fillId="17" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="30" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="17" fontId="14" fillId="17" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -3067,68 +3131,116 @@
     <xf numFmtId="0" fontId="20" fillId="4" borderId="36" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="100" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="101" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="102" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="103" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="104" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="105" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="38" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="103" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="104" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="105" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="65" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="17" fontId="14" fillId="17" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="30" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="17" fontId="14" fillId="17" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="73" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="76" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="78" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="79" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="80" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="33" fillId="18" borderId="52" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -3181,120 +3293,12 @@
     <xf numFmtId="164" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="65" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="73" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="76" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="78" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="79" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="80" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="100" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="101" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="102" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="103" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="104" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="105" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="103" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="104" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="105" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="5">
-    <cellStyle name="20% - Accent2 2" xfId="1"/>
-    <cellStyle name="Comma 2" xfId="4"/>
+    <cellStyle name="20% - Accent2 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+    <cellStyle name="Comma 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
   </cellStyles>
   <dxfs count="60">
@@ -4203,53 +4207,6 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>155370</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>23812</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>631032</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>561695</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Shape 8">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7532368D-E47A-4675-B0B1-9A439F8F0594}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5">
-          <a:alphaModFix/>
-        </a:blip>
-        <a:srcRect b="17423"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="9978026" y="23812"/>
-          <a:ext cx="1666287" cy="537883"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -4549,12 +4506,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A2:Q41"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.5703125" style="16" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="89.42578125" style="26" bestFit="1" customWidth="1"/>
@@ -4576,89 +4533,89 @@
     <col min="18" max="16384" width="8.85546875" style="15"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:17" s="1" customFormat="1">
-      <c r="A2" s="231"/>
-      <c r="B2" s="231"/>
-      <c r="C2" s="231"/>
-      <c r="D2" s="231"/>
-      <c r="E2" s="231"/>
-      <c r="F2" s="231"/>
-      <c r="G2" s="231"/>
-      <c r="H2" s="231"/>
-      <c r="I2" s="231"/>
-    </row>
-    <row r="3" spans="1:17" s="1" customFormat="1">
-      <c r="A3" s="231"/>
-      <c r="B3" s="231"/>
-      <c r="C3" s="231"/>
-      <c r="D3" s="231"/>
-      <c r="E3" s="231"/>
-      <c r="F3" s="231"/>
-      <c r="G3" s="231"/>
-      <c r="H3" s="231"/>
-      <c r="I3" s="231"/>
-    </row>
-    <row r="4" spans="1:17" s="1" customFormat="1">
-      <c r="A4" s="231"/>
-      <c r="B4" s="231"/>
-      <c r="C4" s="231"/>
-      <c r="D4" s="231"/>
-      <c r="E4" s="231"/>
-      <c r="F4" s="231"/>
-      <c r="G4" s="231"/>
-      <c r="H4" s="231"/>
-      <c r="I4" s="231"/>
-    </row>
-    <row r="6" spans="1:17" ht="26.25">
-      <c r="A6" s="238" t="s">
+    <row r="2" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="216"/>
+      <c r="B2" s="216"/>
+      <c r="C2" s="216"/>
+      <c r="D2" s="216"/>
+      <c r="E2" s="216"/>
+      <c r="F2" s="216"/>
+      <c r="G2" s="216"/>
+      <c r="H2" s="216"/>
+      <c r="I2" s="216"/>
+    </row>
+    <row r="3" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="216"/>
+      <c r="B3" s="216"/>
+      <c r="C3" s="216"/>
+      <c r="D3" s="216"/>
+      <c r="E3" s="216"/>
+      <c r="F3" s="216"/>
+      <c r="G3" s="216"/>
+      <c r="H3" s="216"/>
+      <c r="I3" s="216"/>
+    </row>
+    <row r="4" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="216"/>
+      <c r="B4" s="216"/>
+      <c r="C4" s="216"/>
+      <c r="D4" s="216"/>
+      <c r="E4" s="216"/>
+      <c r="F4" s="216"/>
+      <c r="G4" s="216"/>
+      <c r="H4" s="216"/>
+      <c r="I4" s="216"/>
+    </row>
+    <row r="6" spans="1:17" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="A6" s="225" t="s">
         <v>97</v>
       </c>
-      <c r="B6" s="238"/>
-      <c r="C6" s="238"/>
-      <c r="D6" s="238"/>
-      <c r="E6" s="238"/>
-      <c r="F6" s="238"/>
-      <c r="G6" s="238"/>
-      <c r="H6" s="238"/>
-      <c r="I6" s="238"/>
-      <c r="J6" s="238"/>
-      <c r="K6" s="238"/>
-      <c r="L6" s="238"/>
-      <c r="M6" s="238"/>
-      <c r="N6" s="238"/>
-      <c r="O6" s="238"/>
-      <c r="P6" s="238"/>
-      <c r="Q6" s="238"/>
-    </row>
-    <row r="7" spans="1:17" ht="15.75" thickBot="1"/>
-    <row r="8" spans="1:17" s="18" customFormat="1" ht="25.15" customHeight="1" thickTop="1">
+      <c r="B6" s="225"/>
+      <c r="C6" s="225"/>
+      <c r="D6" s="225"/>
+      <c r="E6" s="225"/>
+      <c r="F6" s="225"/>
+      <c r="G6" s="225"/>
+      <c r="H6" s="225"/>
+      <c r="I6" s="225"/>
+      <c r="J6" s="225"/>
+      <c r="K6" s="225"/>
+      <c r="L6" s="225"/>
+      <c r="M6" s="225"/>
+      <c r="N6" s="225"/>
+      <c r="O6" s="225"/>
+      <c r="P6" s="225"/>
+      <c r="Q6" s="225"/>
+    </row>
+    <row r="7" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:17" s="18" customFormat="1" ht="25.15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A8" s="25"/>
-      <c r="B8" s="239" t="s">
+      <c r="B8" s="226" t="s">
         <v>30</v>
       </c>
-      <c r="C8" s="239"/>
-      <c r="D8" s="239"/>
-      <c r="E8" s="239"/>
-      <c r="F8" s="240" t="s">
+      <c r="C8" s="226"/>
+      <c r="D8" s="226"/>
+      <c r="E8" s="226"/>
+      <c r="F8" s="227" t="s">
         <v>31</v>
       </c>
-      <c r="G8" s="240"/>
-      <c r="H8" s="240"/>
-      <c r="I8" s="240"/>
-      <c r="J8" s="240" t="s">
+      <c r="G8" s="227"/>
+      <c r="H8" s="227"/>
+      <c r="I8" s="227"/>
+      <c r="J8" s="227" t="s">
         <v>32</v>
       </c>
-      <c r="K8" s="240"/>
-      <c r="L8" s="240"/>
-      <c r="M8" s="240"/>
-      <c r="N8" s="240" t="s">
+      <c r="K8" s="227"/>
+      <c r="L8" s="227"/>
+      <c r="M8" s="227"/>
+      <c r="N8" s="227" t="s">
         <v>33</v>
       </c>
-      <c r="O8" s="240"/>
-      <c r="P8" s="240"/>
-      <c r="Q8" s="248"/>
-    </row>
-    <row r="9" spans="1:17" s="24" customFormat="1" ht="15.75">
+      <c r="O8" s="227"/>
+      <c r="P8" s="227"/>
+      <c r="Q8" s="235"/>
+    </row>
+    <row r="9" spans="1:17" s="24" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
         <v>17</v>
       </c>
@@ -4711,34 +4668,34 @@
         <v>37</v>
       </c>
     </row>
-    <row r="10" spans="1:17" s="32" customFormat="1" ht="58.15" customHeight="1">
-      <c r="A10" s="241" t="s">
+    <row r="10" spans="1:17" s="32" customFormat="1" ht="58.15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="228" t="s">
         <v>89</v>
       </c>
-      <c r="B10" s="242"/>
-      <c r="C10" s="242"/>
-      <c r="D10" s="242"/>
-      <c r="E10" s="242"/>
-      <c r="F10" s="243" t="s">
+      <c r="B10" s="229"/>
+      <c r="C10" s="229"/>
+      <c r="D10" s="229"/>
+      <c r="E10" s="229"/>
+      <c r="F10" s="230" t="s">
         <v>38</v>
       </c>
-      <c r="G10" s="243"/>
-      <c r="H10" s="243"/>
-      <c r="I10" s="243"/>
-      <c r="J10" s="243" t="s">
+      <c r="G10" s="230"/>
+      <c r="H10" s="230"/>
+      <c r="I10" s="230"/>
+      <c r="J10" s="230" t="s">
         <v>39</v>
       </c>
-      <c r="K10" s="243"/>
-      <c r="L10" s="243"/>
-      <c r="M10" s="243"/>
-      <c r="N10" s="243" t="s">
+      <c r="K10" s="230"/>
+      <c r="L10" s="230"/>
+      <c r="M10" s="230"/>
+      <c r="N10" s="230" t="s">
         <v>40</v>
       </c>
-      <c r="O10" s="243"/>
-      <c r="P10" s="243"/>
-      <c r="Q10" s="244"/>
-    </row>
-    <row r="11" spans="1:17" s="38" customFormat="1" ht="43.9" customHeight="1">
+      <c r="O10" s="230"/>
+      <c r="P10" s="230"/>
+      <c r="Q10" s="231"/>
+    </row>
+    <row r="11" spans="1:17" s="38" customFormat="1" ht="43.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="34">
         <v>1</v>
       </c>
@@ -4777,7 +4734,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="12" spans="1:17" s="38" customFormat="1" ht="50.65" customHeight="1">
+    <row r="12" spans="1:17" s="38" customFormat="1" ht="50.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="39">
         <v>2</v>
       </c>
@@ -4816,7 +4773,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="13" spans="1:17" s="38" customFormat="1" ht="45" customHeight="1">
+    <row r="13" spans="1:17" s="38" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="34">
         <v>3</v>
       </c>
@@ -4861,7 +4818,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:17" s="38" customFormat="1" ht="42" customHeight="1">
+    <row r="14" spans="1:17" s="38" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="39">
         <v>4</v>
       </c>
@@ -4900,7 +4857,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:17" s="38" customFormat="1" ht="36">
+    <row r="15" spans="1:17" s="38" customFormat="1" ht="36" x14ac:dyDescent="0.25">
       <c r="A15" s="34">
         <v>5</v>
       </c>
@@ -4939,7 +4896,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:17" s="38" customFormat="1" ht="36">
+    <row r="16" spans="1:17" s="38" customFormat="1" ht="36" x14ac:dyDescent="0.25">
       <c r="A16" s="39">
         <v>6</v>
       </c>
@@ -4972,7 +4929,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:17" s="38" customFormat="1" ht="55.9" customHeight="1">
+    <row r="17" spans="1:17" s="38" customFormat="1" ht="55.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="34">
         <v>7</v>
       </c>
@@ -5011,7 +4968,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="18" spans="1:17" s="38" customFormat="1" ht="36">
+    <row r="18" spans="1:17" s="38" customFormat="1" ht="36" x14ac:dyDescent="0.25">
       <c r="A18" s="39">
         <v>8</v>
       </c>
@@ -5044,7 +5001,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="19" spans="1:17" s="38" customFormat="1" ht="36">
+    <row r="19" spans="1:17" s="38" customFormat="1" ht="36" x14ac:dyDescent="0.25">
       <c r="A19" s="34">
         <v>9</v>
       </c>
@@ -5083,7 +5040,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="20" spans="1:17" s="38" customFormat="1" ht="36">
+    <row r="20" spans="1:17" s="38" customFormat="1" ht="36" x14ac:dyDescent="0.25">
       <c r="A20" s="34">
         <v>10</v>
       </c>
@@ -5122,7 +5079,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:17" s="33" customFormat="1" ht="20.25">
+    <row r="21" spans="1:17" s="33" customFormat="1" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A21" s="29">
         <v>11</v>
       </c>
@@ -5130,24 +5087,24 @@
         <v>48</v>
       </c>
       <c r="C21" s="31"/>
-      <c r="D21" s="216" t="s">
+      <c r="D21" s="236" t="s">
         <v>93</v>
       </c>
-      <c r="E21" s="217"/>
-      <c r="F21" s="217"/>
-      <c r="G21" s="217"/>
-      <c r="H21" s="217"/>
-      <c r="I21" s="217"/>
-      <c r="J21" s="217"/>
-      <c r="K21" s="217"/>
-      <c r="L21" s="217"/>
-      <c r="M21" s="217"/>
-      <c r="N21" s="217"/>
-      <c r="O21" s="217"/>
-      <c r="P21" s="217"/>
-      <c r="Q21" s="218"/>
-    </row>
-    <row r="22" spans="1:17" s="14" customFormat="1" ht="18">
+      <c r="E21" s="237"/>
+      <c r="F21" s="237"/>
+      <c r="G21" s="237"/>
+      <c r="H21" s="237"/>
+      <c r="I21" s="237"/>
+      <c r="J21" s="237"/>
+      <c r="K21" s="237"/>
+      <c r="L21" s="237"/>
+      <c r="M21" s="237"/>
+      <c r="N21" s="237"/>
+      <c r="O21" s="237"/>
+      <c r="P21" s="237"/>
+      <c r="Q21" s="238"/>
+    </row>
+    <row r="22" spans="1:17" s="14" customFormat="1" ht="18" x14ac:dyDescent="0.25">
       <c r="A22" s="69">
         <v>11.1</v>
       </c>
@@ -5158,7 +5115,7 @@
       <c r="D22" s="69" t="s">
         <v>81</v>
       </c>
-      <c r="E22" s="228" t="s">
+      <c r="E22" s="217" t="s">
         <v>56</v>
       </c>
       <c r="F22" s="35"/>
@@ -5186,7 +5143,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:17" s="14" customFormat="1" ht="18">
+    <row r="23" spans="1:17" s="14" customFormat="1" ht="18" x14ac:dyDescent="0.25">
       <c r="A23" s="69">
         <v>11.2</v>
       </c>
@@ -5197,7 +5154,7 @@
       <c r="D23" s="69" t="s">
         <v>72</v>
       </c>
-      <c r="E23" s="229"/>
+      <c r="E23" s="248"/>
       <c r="F23" s="40" t="s">
         <v>44</v>
       </c>
@@ -5229,7 +5186,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="24" spans="1:17" s="14" customFormat="1" ht="18">
+    <row r="24" spans="1:17" s="14" customFormat="1" ht="18" x14ac:dyDescent="0.25">
       <c r="A24" s="69">
         <v>11.3</v>
       </c>
@@ -5240,7 +5197,7 @@
       <c r="D24" s="69" t="s">
         <v>82</v>
       </c>
-      <c r="E24" s="230"/>
+      <c r="E24" s="218"/>
       <c r="F24" s="35"/>
       <c r="G24" s="35" t="s">
         <v>41</v>
@@ -5266,7 +5223,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="25" spans="1:17" s="14" customFormat="1" ht="36">
+    <row r="25" spans="1:17" s="14" customFormat="1" ht="36" x14ac:dyDescent="0.25">
       <c r="A25" s="69">
         <v>11.4</v>
       </c>
@@ -5277,7 +5234,7 @@
       <c r="D25" s="69" t="s">
         <v>83</v>
       </c>
-      <c r="E25" s="228" t="s">
+      <c r="E25" s="217" t="s">
         <v>80</v>
       </c>
       <c r="F25" s="40"/>
@@ -5305,7 +5262,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="26" spans="1:17" s="14" customFormat="1" ht="18.75" thickBot="1">
+    <row r="26" spans="1:17" s="14" customFormat="1" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="69">
         <v>11.5</v>
       </c>
@@ -5316,7 +5273,7 @@
       <c r="D26" s="69" t="s">
         <v>84</v>
       </c>
-      <c r="E26" s="230"/>
+      <c r="E26" s="218"/>
       <c r="F26" s="45"/>
       <c r="G26" s="45" t="s">
         <v>41</v>
@@ -5342,53 +5299,53 @@
         <v>42</v>
       </c>
     </row>
-    <row r="27" spans="1:17" ht="16.5" thickTop="1" thickBot="1">
-      <c r="A27" s="245"/>
-      <c r="B27" s="246"/>
-      <c r="C27" s="246"/>
-      <c r="D27" s="246"/>
-      <c r="E27" s="246"/>
-      <c r="F27" s="246"/>
-      <c r="G27" s="246"/>
-      <c r="H27" s="246"/>
-      <c r="I27" s="246"/>
-      <c r="J27" s="246"/>
-      <c r="K27" s="246"/>
-      <c r="L27" s="246"/>
-      <c r="M27" s="246"/>
-      <c r="N27" s="246"/>
-      <c r="O27" s="246"/>
-      <c r="P27" s="246"/>
-      <c r="Q27" s="247"/>
-    </row>
-    <row r="28" spans="1:17" s="32" customFormat="1" ht="21" thickTop="1">
-      <c r="A28" s="235" t="s">
+    <row r="27" spans="1:17" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="232"/>
+      <c r="B27" s="233"/>
+      <c r="C27" s="233"/>
+      <c r="D27" s="233"/>
+      <c r="E27" s="233"/>
+      <c r="F27" s="233"/>
+      <c r="G27" s="233"/>
+      <c r="H27" s="233"/>
+      <c r="I27" s="233"/>
+      <c r="J27" s="233"/>
+      <c r="K27" s="233"/>
+      <c r="L27" s="233"/>
+      <c r="M27" s="233"/>
+      <c r="N27" s="233"/>
+      <c r="O27" s="233"/>
+      <c r="P27" s="233"/>
+      <c r="Q27" s="234"/>
+    </row>
+    <row r="28" spans="1:17" s="32" customFormat="1" ht="21" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="222" t="s">
         <v>90</v>
       </c>
-      <c r="B28" s="236"/>
-      <c r="C28" s="236"/>
-      <c r="D28" s="236"/>
-      <c r="E28" s="237"/>
-      <c r="F28" s="225" t="s">
+      <c r="B28" s="223"/>
+      <c r="C28" s="223"/>
+      <c r="D28" s="223"/>
+      <c r="E28" s="224"/>
+      <c r="F28" s="245" t="s">
         <v>45</v>
       </c>
-      <c r="G28" s="226"/>
-      <c r="H28" s="226"/>
-      <c r="I28" s="227"/>
-      <c r="J28" s="222" t="s">
+      <c r="G28" s="246"/>
+      <c r="H28" s="246"/>
+      <c r="I28" s="247"/>
+      <c r="J28" s="242" t="s">
         <v>45</v>
       </c>
-      <c r="K28" s="223"/>
-      <c r="L28" s="223"/>
-      <c r="M28" s="224"/>
-      <c r="N28" s="219" t="s">
+      <c r="K28" s="243"/>
+      <c r="L28" s="243"/>
+      <c r="M28" s="244"/>
+      <c r="N28" s="239" t="s">
         <v>45</v>
       </c>
-      <c r="O28" s="220"/>
-      <c r="P28" s="220"/>
-      <c r="Q28" s="221"/>
-    </row>
-    <row r="29" spans="1:17" s="38" customFormat="1" ht="55.5" customHeight="1">
+      <c r="O28" s="240"/>
+      <c r="P28" s="240"/>
+      <c r="Q28" s="241"/>
+    </row>
+    <row r="29" spans="1:17" s="38" customFormat="1" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="69">
         <v>12</v>
       </c>
@@ -5427,7 +5384,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="30" spans="1:17" s="38" customFormat="1" ht="55.5" customHeight="1">
+    <row r="30" spans="1:17" s="38" customFormat="1" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="69">
         <v>13</v>
       </c>
@@ -5466,7 +5423,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="31" spans="1:17" s="38" customFormat="1" ht="55.5" customHeight="1">
+    <row r="31" spans="1:17" s="38" customFormat="1" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="69">
         <v>14</v>
       </c>
@@ -5499,7 +5456,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="32" spans="1:17" s="14" customFormat="1" ht="55.5" customHeight="1">
+    <row r="32" spans="1:17" s="14" customFormat="1" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="69">
         <v>15</v>
       </c>
@@ -5532,7 +5489,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="33" spans="1:17" s="14" customFormat="1" ht="55.5" customHeight="1">
+    <row r="33" spans="1:17" s="14" customFormat="1" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="69">
         <v>16</v>
       </c>
@@ -5571,7 +5528,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="34" spans="1:17" s="13" customFormat="1" ht="20.25">
+    <row r="34" spans="1:17" s="13" customFormat="1" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A34" s="29">
         <v>17</v>
       </c>
@@ -5579,24 +5536,24 @@
         <v>23</v>
       </c>
       <c r="C34" s="31"/>
-      <c r="D34" s="216" t="s">
+      <c r="D34" s="236" t="s">
         <v>93</v>
       </c>
-      <c r="E34" s="217"/>
-      <c r="F34" s="217"/>
-      <c r="G34" s="217"/>
-      <c r="H34" s="217"/>
-      <c r="I34" s="217"/>
-      <c r="J34" s="217"/>
-      <c r="K34" s="217"/>
-      <c r="L34" s="217"/>
-      <c r="M34" s="217"/>
-      <c r="N34" s="217"/>
-      <c r="O34" s="217"/>
-      <c r="P34" s="217"/>
-      <c r="Q34" s="218"/>
-    </row>
-    <row r="35" spans="1:17" s="14" customFormat="1" ht="41.65" customHeight="1">
+      <c r="E34" s="237"/>
+      <c r="F34" s="237"/>
+      <c r="G34" s="237"/>
+      <c r="H34" s="237"/>
+      <c r="I34" s="237"/>
+      <c r="J34" s="237"/>
+      <c r="K34" s="237"/>
+      <c r="L34" s="237"/>
+      <c r="M34" s="237"/>
+      <c r="N34" s="237"/>
+      <c r="O34" s="237"/>
+      <c r="P34" s="237"/>
+      <c r="Q34" s="238"/>
+    </row>
+    <row r="35" spans="1:17" s="14" customFormat="1" ht="41.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="69">
         <v>17.100000000000001</v>
       </c>
@@ -5607,7 +5564,7 @@
       <c r="D35" s="69" t="s">
         <v>52</v>
       </c>
-      <c r="E35" s="232" t="s">
+      <c r="E35" s="219" t="s">
         <v>116</v>
       </c>
       <c r="F35" s="59"/>
@@ -5635,7 +5592,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="36" spans="1:17" s="14" customFormat="1" ht="46.15" customHeight="1">
+    <row r="36" spans="1:17" s="14" customFormat="1" ht="46.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="69">
         <v>17.2</v>
       </c>
@@ -5646,7 +5603,7 @@
       <c r="D36" s="69" t="s">
         <v>53</v>
       </c>
-      <c r="E36" s="233"/>
+      <c r="E36" s="220"/>
       <c r="F36" s="61"/>
       <c r="G36" s="40" t="s">
         <v>77</v>
@@ -5672,7 +5629,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="37" spans="1:17" s="14" customFormat="1" ht="40.5" customHeight="1">
+    <row r="37" spans="1:17" s="14" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="69">
         <v>17.3</v>
       </c>
@@ -5683,7 +5640,7 @@
       <c r="D37" s="69" t="s">
         <v>51</v>
       </c>
-      <c r="E37" s="234"/>
+      <c r="E37" s="221"/>
       <c r="F37" s="59" t="s">
         <v>47</v>
       </c>
@@ -5715,7 +5672,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="38" spans="1:17" s="14" customFormat="1" ht="40.5" customHeight="1">
+    <row r="38" spans="1:17" s="14" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="69">
         <v>17.399999999999999</v>
       </c>
@@ -5726,7 +5683,7 @@
       <c r="D38" s="69" t="s">
         <v>54</v>
       </c>
-      <c r="E38" s="232" t="s">
+      <c r="E38" s="219" t="s">
         <v>79</v>
       </c>
       <c r="F38" s="61"/>
@@ -5754,7 +5711,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="39" spans="1:17" s="14" customFormat="1" ht="40.5" customHeight="1">
+    <row r="39" spans="1:17" s="14" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="69">
         <v>17.5</v>
       </c>
@@ -5765,7 +5722,7 @@
       <c r="D39" s="69" t="s">
         <v>55</v>
       </c>
-      <c r="E39" s="233"/>
+      <c r="E39" s="220"/>
       <c r="F39" s="59"/>
       <c r="G39" s="35" t="s">
         <v>77</v>
@@ -5791,7 +5748,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="40" spans="1:17" s="14" customFormat="1" ht="40.5" customHeight="1" thickBot="1">
+    <row r="40" spans="1:17" s="14" customFormat="1" ht="40.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="69">
         <v>17.600000000000001</v>
       </c>
@@ -5802,7 +5759,7 @@
       <c r="D40" s="69" t="s">
         <v>85</v>
       </c>
-      <c r="E40" s="234"/>
+      <c r="E40" s="221"/>
       <c r="F40" s="63"/>
       <c r="G40" s="64" t="s">
         <v>77</v>
@@ -5828,9 +5785,14 @@
         <v>42</v>
       </c>
     </row>
-    <row r="41" spans="1:17" ht="15.75" thickTop="1"/>
+    <row r="41" spans="1:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="D34:Q34"/>
+    <mergeCell ref="N28:Q28"/>
+    <mergeCell ref="J28:M28"/>
+    <mergeCell ref="F28:I28"/>
+    <mergeCell ref="E22:E24"/>
     <mergeCell ref="A2:I4"/>
     <mergeCell ref="E25:E26"/>
     <mergeCell ref="E35:E37"/>
@@ -5847,11 +5809,6 @@
     <mergeCell ref="A27:Q27"/>
     <mergeCell ref="N8:Q8"/>
     <mergeCell ref="D21:Q21"/>
-    <mergeCell ref="D34:Q34"/>
-    <mergeCell ref="N28:Q28"/>
-    <mergeCell ref="J28:M28"/>
-    <mergeCell ref="F28:I28"/>
-    <mergeCell ref="E22:E24"/>
   </mergeCells>
   <pageMargins left="0.37037037037037002" right="0.51136363636363602" top="0.43154761904761901" bottom="0.64583333333333304" header="0.5" footer="0.5"/>
   <pageSetup paperSize="256" scale="74" fitToHeight="0" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
@@ -5866,13 +5823,13 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor rgb="FF00B050"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:X40"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.5703125" style="1" customWidth="1"/>
     <col min="2" max="2" width="12.5703125" style="9" customWidth="1"/>
@@ -5896,7 +5853,7 @@
     <col min="20" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:24" s="75" customFormat="1" ht="34.35" hidden="1" customHeight="1" thickBot="1">
+    <row r="1" spans="2:24" s="75" customFormat="1" ht="34.35" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B1" s="84" t="s">
         <v>103</v>
       </c>
@@ -5922,13 +5879,13 @@
         <v>2020</v>
       </c>
       <c r="J1" s="88"/>
-      <c r="K1" s="266" t="s">
+      <c r="K1" s="262" t="s">
         <v>108</v>
       </c>
-      <c r="L1" s="267"/>
-      <c r="M1" s="267"/>
-      <c r="N1" s="267"/>
-      <c r="O1" s="268"/>
+      <c r="L1" s="263"/>
+      <c r="M1" s="263"/>
+      <c r="N1" s="263"/>
+      <c r="O1" s="264"/>
       <c r="P1" s="89"/>
       <c r="Q1" s="90">
         <f>DATE(I1,G1,"01")</f>
@@ -5950,46 +5907,46 @@
       </c>
       <c r="X1" s="74"/>
     </row>
-    <row r="2" spans="2:24" s="77" customFormat="1" ht="34.35" hidden="1" customHeight="1" thickBot="1">
-      <c r="B2" s="275" t="s">
+    <row r="2" spans="2:24" s="77" customFormat="1" ht="34.35" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B2" s="271" t="s">
         <v>109</v>
       </c>
-      <c r="C2" s="276"/>
-      <c r="D2" s="276"/>
-      <c r="E2" s="276"/>
-      <c r="F2" s="276"/>
-      <c r="G2" s="276"/>
-      <c r="H2" s="276"/>
-      <c r="I2" s="276"/>
-      <c r="J2" s="276"/>
-      <c r="K2" s="276"/>
-      <c r="L2" s="276"/>
-      <c r="M2" s="276"/>
-      <c r="N2" s="276"/>
-      <c r="O2" s="276"/>
-      <c r="P2" s="276"/>
-      <c r="Q2" s="276"/>
-      <c r="R2" s="276"/>
-      <c r="S2" s="277"/>
+      <c r="C2" s="272"/>
+      <c r="D2" s="272"/>
+      <c r="E2" s="272"/>
+      <c r="F2" s="272"/>
+      <c r="G2" s="272"/>
+      <c r="H2" s="272"/>
+      <c r="I2" s="272"/>
+      <c r="J2" s="272"/>
+      <c r="K2" s="272"/>
+      <c r="L2" s="272"/>
+      <c r="M2" s="272"/>
+      <c r="N2" s="272"/>
+      <c r="O2" s="272"/>
+      <c r="P2" s="272"/>
+      <c r="Q2" s="272"/>
+      <c r="R2" s="272"/>
+      <c r="S2" s="273"/>
       <c r="T2" s="76"/>
       <c r="W2" s="73">
         <v>1</v>
       </c>
       <c r="X2" s="78"/>
     </row>
-    <row r="3" spans="2:24" s="77" customFormat="1" ht="48" customHeight="1" thickBot="1">
+    <row r="3" spans="2:24" s="77" customFormat="1" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B3" s="151"/>
       <c r="C3" s="152"/>
       <c r="D3" s="152"/>
       <c r="E3" s="152"/>
       <c r="F3" s="153"/>
       <c r="G3" s="92"/>
-      <c r="H3" s="280" t="str">
+      <c r="H3" s="276" t="str">
         <f>IF(LEN(L8&amp;L26)&lt;1,"","Form Has Data Errors, Please correct before submitting or uploading")</f>
         <v/>
       </c>
-      <c r="I3" s="281"/>
-      <c r="J3" s="282"/>
+      <c r="I3" s="277"/>
+      <c r="J3" s="278"/>
       <c r="K3" s="92"/>
       <c r="L3" s="92"/>
       <c r="M3" s="158"/>
@@ -6003,19 +5960,19 @@
       <c r="W3" s="73"/>
       <c r="X3" s="78"/>
     </row>
-    <row r="4" spans="2:24" s="77" customFormat="1" ht="24" customHeight="1" thickBot="1">
-      <c r="B4" s="272" t="str">
+    <row r="4" spans="2:24" s="77" customFormat="1" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B4" s="268" t="str">
         <f>B1&amp;" : "&amp;C1&amp;"                                                           MFLCode : "&amp;E1&amp;"                                                    Reporting Month :   "&amp;G1&amp;"                                             Reporting Year: "&amp;I1</f>
         <v>Health Facility : Likii Dispensary                                                           MFLCode : 15035                                                    Reporting Month :   02                                             Reporting Year: 2020</v>
       </c>
-      <c r="C4" s="273"/>
-      <c r="D4" s="273"/>
-      <c r="E4" s="273"/>
-      <c r="F4" s="274"/>
+      <c r="C4" s="269"/>
+      <c r="D4" s="269"/>
+      <c r="E4" s="269"/>
+      <c r="F4" s="270"/>
       <c r="G4" s="93"/>
-      <c r="H4" s="283"/>
-      <c r="I4" s="284"/>
-      <c r="J4" s="285"/>
+      <c r="H4" s="279"/>
+      <c r="I4" s="280"/>
+      <c r="J4" s="281"/>
       <c r="K4" s="94"/>
       <c r="L4" s="94"/>
       <c r="M4" s="94"/>
@@ -6037,20 +5994,20 @@
       </c>
       <c r="X4" s="78"/>
     </row>
-    <row r="5" spans="2:24" s="81" customFormat="1" ht="30.75" customHeight="1" thickBot="1">
-      <c r="B5" s="278" t="s">
+    <row r="5" spans="2:24" s="81" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B5" s="274" t="s">
         <v>110</v>
       </c>
-      <c r="C5" s="279"/>
-      <c r="D5" s="269" t="s">
+      <c r="C5" s="275"/>
+      <c r="D5" s="265" t="s">
         <v>111</v>
       </c>
-      <c r="E5" s="270"/>
-      <c r="F5" s="271"/>
+      <c r="E5" s="266"/>
+      <c r="F5" s="267"/>
       <c r="G5" s="97"/>
-      <c r="H5" s="286"/>
-      <c r="I5" s="287"/>
-      <c r="J5" s="288"/>
+      <c r="H5" s="282"/>
+      <c r="I5" s="283"/>
+      <c r="J5" s="284"/>
       <c r="K5" s="97"/>
       <c r="L5" s="97"/>
       <c r="M5" s="97"/>
@@ -6068,11 +6025,11 @@
       </c>
       <c r="X5" s="80"/>
     </row>
-    <row r="6" spans="2:24" s="2" customFormat="1" ht="27.75" customHeight="1" thickBot="1">
-      <c r="B6" s="249" t="s">
+    <row r="6" spans="2:24" s="2" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="285" t="s">
         <v>98</v>
       </c>
-      <c r="C6" s="250"/>
+      <c r="C6" s="286"/>
       <c r="D6" s="98" t="s">
         <v>115</v>
       </c>
@@ -6081,12 +6038,12 @@
         <v>43497</v>
       </c>
       <c r="F6" s="160"/>
-      <c r="G6" s="256"/>
-      <c r="H6" s="253" t="s">
+      <c r="G6" s="292"/>
+      <c r="H6" s="289" t="s">
         <v>86</v>
       </c>
-      <c r="I6" s="254"/>
-      <c r="J6" s="255"/>
+      <c r="I6" s="290"/>
+      <c r="J6" s="291"/>
       <c r="K6" s="100"/>
       <c r="L6" s="100"/>
       <c r="M6" s="100"/>
@@ -6097,7 +6054,7 @@
       <c r="R6" s="100"/>
       <c r="S6" s="100"/>
     </row>
-    <row r="7" spans="2:24" s="70" customFormat="1" ht="19.5" customHeight="1" thickBot="1">
+    <row r="7" spans="2:24" s="70" customFormat="1" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="101" t="s">
         <v>17</v>
       </c>
@@ -6113,7 +6070,7 @@
       <c r="F7" s="186" t="s">
         <v>2</v>
       </c>
-      <c r="G7" s="256"/>
+      <c r="G7" s="292"/>
       <c r="H7" s="168" t="s">
         <v>0</v>
       </c>
@@ -6139,7 +6096,7 @@
       <c r="R7" s="106"/>
       <c r="S7" s="106"/>
     </row>
-    <row r="8" spans="2:24" s="3" customFormat="1" ht="25.5" customHeight="1">
+    <row r="8" spans="2:24" s="3" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="107">
         <v>1</v>
       </c>
@@ -6152,7 +6109,7 @@
         <f>IFERROR(D8/E8,)</f>
         <v>0</v>
       </c>
-      <c r="G8" s="256"/>
+      <c r="G8" s="292"/>
       <c r="H8" s="164"/>
       <c r="I8" s="165" t="s">
         <v>41</v>
@@ -6162,12 +6119,12 @@
         <f>IF(D8&gt;E8,"*Numerator for "&amp;C8&amp;" Cannot be more than Denominator"&amp;CHAR(10),"")</f>
         <v/>
       </c>
-      <c r="L8" s="292" t="str">
+      <c r="L8" s="252" t="str">
         <f>CONCATENATE(K8,K9,K10,K11,K12,K13,K14,K15,K16,K17,K18,K19,K20,K21,K22,K23,K24)</f>
         <v/>
       </c>
       <c r="M8" s="170"/>
-      <c r="N8" s="289" t="str">
+      <c r="N8" s="249" t="str">
         <f>CONCATENATE(M8,M9,M10,M11,M12,M13,M14,M15,M16,M17,M18,M19,M20,M21,M22,M23)</f>
         <v/>
       </c>
@@ -6177,7 +6134,7 @@
       <c r="R8" s="111"/>
       <c r="S8" s="111"/>
     </row>
-    <row r="9" spans="2:24" s="4" customFormat="1" ht="25.5" customHeight="1">
+    <row r="9" spans="2:24" s="4" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="107">
         <v>2</v>
       </c>
@@ -6193,7 +6150,7 @@
         <f t="shared" ref="F9:F23" si="0">IFERROR(D9/E9,)</f>
         <v>0</v>
       </c>
-      <c r="G9" s="256"/>
+      <c r="G9" s="292"/>
       <c r="H9" s="108"/>
       <c r="I9" s="109" t="s">
         <v>41</v>
@@ -6203,16 +6160,16 @@
         <f t="shared" ref="K9:K23" si="1">IF(D9&gt;E9,"*Numerator for "&amp;C9&amp;" Cannot be more than Denominator"&amp;CHAR(10),"")</f>
         <v/>
       </c>
-      <c r="L9" s="293"/>
+      <c r="L9" s="253"/>
       <c r="M9" s="170"/>
-      <c r="N9" s="290"/>
+      <c r="N9" s="250"/>
       <c r="O9" s="174"/>
       <c r="P9" s="112"/>
       <c r="Q9" s="112"/>
       <c r="R9" s="112"/>
       <c r="S9" s="112"/>
     </row>
-    <row r="10" spans="2:24" s="3" customFormat="1" ht="25.5" customHeight="1">
+    <row r="10" spans="2:24" s="3" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="107">
         <v>3</v>
       </c>
@@ -6228,7 +6185,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G10" s="256"/>
+      <c r="G10" s="292"/>
       <c r="H10" s="113" t="s">
         <v>43</v>
       </c>
@@ -6240,19 +6197,19 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="L10" s="293"/>
+      <c r="L10" s="253"/>
       <c r="M10" s="170" t="str">
         <f>IF(E10&gt;0,IF(D10/E10&lt;0.85,"*Early Testing Rate is below 85%"&amp;CHAR(10),""),"")</f>
         <v/>
       </c>
-      <c r="N10" s="290"/>
+      <c r="N10" s="250"/>
       <c r="O10" s="173"/>
       <c r="P10" s="111"/>
       <c r="Q10" s="111"/>
       <c r="R10" s="111"/>
       <c r="S10" s="111"/>
     </row>
-    <row r="11" spans="2:24" s="3" customFormat="1" ht="25.5" customHeight="1">
+    <row r="11" spans="2:24" s="3" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="107">
         <v>4</v>
       </c>
@@ -6268,7 +6225,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G11" s="256"/>
+      <c r="G11" s="292"/>
       <c r="H11" s="108"/>
       <c r="I11" s="114" t="s">
         <v>43</v>
@@ -6278,16 +6235,16 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="L11" s="293"/>
+      <c r="L11" s="253"/>
       <c r="M11" s="170"/>
-      <c r="N11" s="290"/>
+      <c r="N11" s="250"/>
       <c r="O11" s="173"/>
       <c r="P11" s="111"/>
       <c r="Q11" s="111"/>
       <c r="R11" s="111"/>
       <c r="S11" s="111"/>
     </row>
-    <row r="12" spans="2:24" s="3" customFormat="1" ht="25.5" customHeight="1">
+    <row r="12" spans="2:24" s="3" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="107">
         <v>5</v>
       </c>
@@ -6303,7 +6260,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G12" s="256"/>
+      <c r="G12" s="292"/>
       <c r="H12" s="115" t="s">
         <v>91</v>
       </c>
@@ -6315,19 +6272,19 @@
         <f>IF(D12&gt;E12,"*Numerator for HEI tested with First DNA PCR at 6-8wks or at First contact and results available between 0 and 12 months Cannot be more than Denominator"&amp;CHAR(10)&amp;CHAR(10),"")</f>
         <v/>
       </c>
-      <c r="L12" s="293"/>
+      <c r="L12" s="253"/>
       <c r="M12" s="170" t="str">
         <f>IF(E12&gt;0,IF(D12/E12&lt;0.95,"*Testing Rate is below 95%"&amp;CHAR(10),""),"")</f>
         <v/>
       </c>
-      <c r="N12" s="290"/>
+      <c r="N12" s="250"/>
       <c r="O12" s="175"/>
       <c r="P12" s="111"/>
       <c r="Q12" s="111"/>
       <c r="R12" s="111"/>
       <c r="S12" s="111"/>
     </row>
-    <row r="13" spans="2:24" s="3" customFormat="1" ht="25.5" customHeight="1">
+    <row r="13" spans="2:24" s="3" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="107">
         <v>6</v>
       </c>
@@ -6343,7 +6300,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G13" s="256"/>
+      <c r="G13" s="292"/>
       <c r="H13" s="116"/>
       <c r="I13" s="117"/>
       <c r="J13" s="110"/>
@@ -6351,16 +6308,16 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="L13" s="293"/>
+      <c r="L13" s="253"/>
       <c r="M13" s="170"/>
-      <c r="N13" s="290"/>
+      <c r="N13" s="250"/>
       <c r="O13" s="173"/>
       <c r="P13" s="111"/>
       <c r="Q13" s="111"/>
       <c r="R13" s="111"/>
       <c r="S13" s="111"/>
     </row>
-    <row r="14" spans="2:24" s="3" customFormat="1" ht="25.5" customHeight="1">
+    <row r="14" spans="2:24" s="3" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="107">
         <v>7</v>
       </c>
@@ -6376,7 +6333,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G14" s="256"/>
+      <c r="G14" s="292"/>
       <c r="H14" s="118" t="s">
         <v>44</v>
       </c>
@@ -6388,16 +6345,16 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="L14" s="293"/>
+      <c r="L14" s="253"/>
       <c r="M14" s="170"/>
-      <c r="N14" s="290"/>
+      <c r="N14" s="250"/>
       <c r="O14" s="173"/>
       <c r="P14" s="111"/>
       <c r="Q14" s="111"/>
       <c r="R14" s="111"/>
       <c r="S14" s="111"/>
     </row>
-    <row r="15" spans="2:24" s="3" customFormat="1" ht="25.5" customHeight="1">
+    <row r="15" spans="2:24" s="3" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="107">
         <v>8</v>
       </c>
@@ -6413,7 +6370,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G15" s="256"/>
+      <c r="G15" s="292"/>
       <c r="H15" s="108"/>
       <c r="I15" s="117"/>
       <c r="J15" s="110"/>
@@ -6421,19 +6378,19 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="L15" s="293"/>
+      <c r="L15" s="253"/>
       <c r="M15" s="170" t="str">
         <f>IF(E15&gt;0,IF(D15/E15&lt;0.85,"*Exclusive Breastfeeding Rate at 6 months is below 85%"&amp;CHAR(10),""),"")</f>
         <v/>
       </c>
-      <c r="N15" s="290"/>
+      <c r="N15" s="250"/>
       <c r="O15" s="173"/>
       <c r="P15" s="111"/>
       <c r="Q15" s="111"/>
       <c r="R15" s="111"/>
       <c r="S15" s="111"/>
     </row>
-    <row r="16" spans="2:24" s="3" customFormat="1" ht="25.5" customHeight="1">
+    <row r="16" spans="2:24" s="3" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="107">
         <v>9</v>
       </c>
@@ -6449,7 +6406,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G16" s="256"/>
+      <c r="G16" s="292"/>
       <c r="H16" s="108"/>
       <c r="I16" s="119" t="s">
         <v>44</v>
@@ -6459,19 +6416,19 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="L16" s="293"/>
+      <c r="L16" s="253"/>
       <c r="M16" s="170" t="str">
         <f>IF(E16&gt;0,IF(D16/E16&lt;0.95,"*Linkage Rate amongest positive infants identified between 0 and 12 months is below 95%"&amp;CHAR(10),""),"")</f>
         <v/>
       </c>
-      <c r="N16" s="290"/>
+      <c r="N16" s="250"/>
       <c r="O16" s="175"/>
       <c r="P16" s="111"/>
       <c r="Q16" s="111"/>
       <c r="R16" s="111"/>
       <c r="S16" s="111"/>
     </row>
-    <row r="17" spans="2:19" s="3" customFormat="1" ht="25.5" customHeight="1">
+    <row r="17" spans="2:19" s="3" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="107">
         <v>10</v>
       </c>
@@ -6487,7 +6444,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G17" s="256"/>
+      <c r="G17" s="292"/>
       <c r="H17" s="108"/>
       <c r="I17" s="119" t="s">
         <v>44</v>
@@ -6497,16 +6454,16 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="L17" s="293"/>
+      <c r="L17" s="253"/>
       <c r="M17" s="170"/>
-      <c r="N17" s="290"/>
+      <c r="N17" s="250"/>
       <c r="O17" s="173"/>
       <c r="P17" s="111"/>
       <c r="Q17" s="111"/>
       <c r="R17" s="111"/>
       <c r="S17" s="111"/>
     </row>
-    <row r="18" spans="2:19" ht="18.75" customHeight="1">
+    <row r="18" spans="2:19" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="150">
         <v>11</v>
       </c>
@@ -6516,7 +6473,7 @@
       <c r="D18" s="193"/>
       <c r="E18" s="187"/>
       <c r="F18" s="194"/>
-      <c r="G18" s="256"/>
+      <c r="G18" s="292"/>
       <c r="H18" s="120"/>
       <c r="I18" s="121"/>
       <c r="J18" s="122"/>
@@ -6524,16 +6481,16 @@
         <f>IF(D12&lt;E11,"*Numerator for "&amp;C12&amp;" Cannot be less than Denominator for "&amp;C11&amp;CHAR(10)&amp;CHAR(10),"")</f>
         <v/>
       </c>
-      <c r="L18" s="293"/>
+      <c r="L18" s="253"/>
       <c r="M18" s="170"/>
-      <c r="N18" s="290"/>
+      <c r="N18" s="250"/>
       <c r="O18" s="176"/>
       <c r="P18" s="123"/>
       <c r="Q18" s="123"/>
       <c r="R18" s="123"/>
       <c r="S18" s="123"/>
     </row>
-    <row r="19" spans="2:19" s="3" customFormat="1" ht="25.5" customHeight="1">
+    <row r="19" spans="2:19" s="3" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="107">
         <v>11.1</v>
       </c>
@@ -6549,7 +6506,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G19" s="256"/>
+      <c r="G19" s="292"/>
       <c r="H19" s="108"/>
       <c r="I19" s="109" t="s">
         <v>41</v>
@@ -6559,16 +6516,16 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="L19" s="293"/>
+      <c r="L19" s="253"/>
       <c r="M19" s="170"/>
-      <c r="N19" s="290"/>
+      <c r="N19" s="250"/>
       <c r="O19" s="173"/>
       <c r="P19" s="111"/>
       <c r="Q19" s="111"/>
       <c r="R19" s="111"/>
       <c r="S19" s="111"/>
     </row>
-    <row r="20" spans="2:19" s="3" customFormat="1" ht="25.5" customHeight="1">
+    <row r="20" spans="2:19" s="3" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="107">
         <v>11.2</v>
       </c>
@@ -6587,7 +6544,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G20" s="256"/>
+      <c r="G20" s="292"/>
       <c r="H20" s="118" t="s">
         <v>44</v>
       </c>
@@ -6599,19 +6556,19 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="L20" s="293"/>
+      <c r="L20" s="253"/>
       <c r="M20" s="170" t="str">
         <f>IF(E20&gt;0,IF(D20/E20&gt;0.05,"*EID Mother To Child Transmission rate is above 5%"&amp;CHAR(10),""),"")</f>
         <v/>
       </c>
-      <c r="N20" s="290"/>
+      <c r="N20" s="250"/>
       <c r="O20" s="173"/>
       <c r="P20" s="111"/>
       <c r="Q20" s="111"/>
       <c r="R20" s="111"/>
       <c r="S20" s="111"/>
     </row>
-    <row r="21" spans="2:19" s="3" customFormat="1" ht="25.5" customHeight="1">
+    <row r="21" spans="2:19" s="3" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="107">
         <v>11.3</v>
       </c>
@@ -6627,7 +6584,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G21" s="256"/>
+      <c r="G21" s="292"/>
       <c r="H21" s="108"/>
       <c r="I21" s="109" t="s">
         <v>41</v>
@@ -6637,16 +6594,16 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="L21" s="293"/>
+      <c r="L21" s="253"/>
       <c r="M21" s="170"/>
-      <c r="N21" s="290"/>
+      <c r="N21" s="250"/>
       <c r="O21" s="173"/>
       <c r="P21" s="111"/>
       <c r="Q21" s="111"/>
       <c r="R21" s="111"/>
       <c r="S21" s="111"/>
     </row>
-    <row r="22" spans="2:19" s="3" customFormat="1" ht="25.5" customHeight="1">
+    <row r="22" spans="2:19" s="3" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="107">
         <v>11.4</v>
       </c>
@@ -6662,7 +6619,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G22" s="256"/>
+      <c r="G22" s="292"/>
       <c r="H22" s="108"/>
       <c r="I22" s="109" t="s">
         <v>41</v>
@@ -6672,16 +6629,16 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="L22" s="293"/>
+      <c r="L22" s="253"/>
       <c r="M22" s="170"/>
-      <c r="N22" s="290"/>
+      <c r="N22" s="250"/>
       <c r="O22" s="173"/>
       <c r="P22" s="111"/>
       <c r="Q22" s="111"/>
       <c r="R22" s="111"/>
       <c r="S22" s="111"/>
     </row>
-    <row r="23" spans="2:19" s="3" customFormat="1" ht="25.5" customHeight="1" thickBot="1">
+    <row r="23" spans="2:19" s="3" customFormat="1" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="157">
         <v>11.5</v>
       </c>
@@ -6697,7 +6654,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G23" s="256"/>
+      <c r="G23" s="292"/>
       <c r="H23" s="126"/>
       <c r="I23" s="127" t="s">
         <v>41</v>
@@ -6707,27 +6664,27 @@
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="L23" s="294"/>
+      <c r="L23" s="254"/>
       <c r="M23" s="170"/>
-      <c r="N23" s="291"/>
+      <c r="N23" s="251"/>
       <c r="O23" s="173"/>
       <c r="P23" s="111"/>
       <c r="Q23" s="111"/>
       <c r="R23" s="111"/>
       <c r="S23" s="111"/>
     </row>
-    <row r="24" spans="2:19" ht="16.5" customHeight="1">
-      <c r="B24" s="257" t="s">
+    <row r="24" spans="2:19" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="293" t="s">
         <v>80</v>
       </c>
-      <c r="C24" s="258"/>
-      <c r="D24" s="259"/>
-      <c r="E24" s="259"/>
-      <c r="F24" s="260"/>
-      <c r="G24" s="256"/>
-      <c r="H24" s="264"/>
-      <c r="I24" s="264"/>
-      <c r="J24" s="264"/>
+      <c r="C24" s="294"/>
+      <c r="D24" s="295"/>
+      <c r="E24" s="295"/>
+      <c r="F24" s="296"/>
+      <c r="G24" s="292"/>
+      <c r="H24" s="300"/>
+      <c r="I24" s="300"/>
+      <c r="J24" s="300"/>
       <c r="K24" s="123" t="str">
         <f>IF(SUM(D19:D23)&lt;&gt;E19,"* Sum of Numerator  11.1,11.2,11.3,11.4 and 11.5 should be equal to Denominator for 11.1","")</f>
         <v/>
@@ -6741,16 +6698,16 @@
       <c r="R24" s="123"/>
       <c r="S24" s="123"/>
     </row>
-    <row r="25" spans="2:19" ht="9.75" customHeight="1" thickBot="1">
-      <c r="B25" s="261"/>
-      <c r="C25" s="262"/>
-      <c r="D25" s="262"/>
-      <c r="E25" s="262"/>
-      <c r="F25" s="263"/>
-      <c r="G25" s="256"/>
-      <c r="H25" s="264"/>
-      <c r="I25" s="264"/>
-      <c r="J25" s="264"/>
+    <row r="25" spans="2:19" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="297"/>
+      <c r="C25" s="298"/>
+      <c r="D25" s="298"/>
+      <c r="E25" s="298"/>
+      <c r="F25" s="299"/>
+      <c r="G25" s="292"/>
+      <c r="H25" s="300"/>
+      <c r="I25" s="300"/>
+      <c r="J25" s="300"/>
       <c r="K25" s="123"/>
       <c r="L25" s="123"/>
       <c r="M25" s="123"/>
@@ -6761,11 +6718,11 @@
       <c r="R25" s="123"/>
       <c r="S25" s="123"/>
     </row>
-    <row r="26" spans="2:19" s="5" customFormat="1" ht="32.25" customHeight="1" thickBot="1">
-      <c r="B26" s="251" t="s">
+    <row r="26" spans="2:19" s="5" customFormat="1" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="287" t="s">
         <v>90</v>
       </c>
-      <c r="C26" s="252"/>
+      <c r="C26" s="288"/>
       <c r="D26" s="129" t="s">
         <v>115</v>
       </c>
@@ -6774,19 +6731,19 @@
         <v>43132</v>
       </c>
       <c r="F26" s="161"/>
-      <c r="G26" s="256"/>
-      <c r="H26" s="295" t="s">
+      <c r="G26" s="292"/>
+      <c r="H26" s="255" t="s">
         <v>86</v>
       </c>
-      <c r="I26" s="296"/>
-      <c r="J26" s="297"/>
+      <c r="I26" s="256"/>
+      <c r="J26" s="257"/>
       <c r="K26" s="131"/>
-      <c r="L26" s="299" t="str">
+      <c r="L26" s="259" t="str">
         <f>CONCATENATE(K28,K29,K30,K31,K32,K33,K34,K35,K36,K37,K38,K39)</f>
         <v/>
       </c>
       <c r="M26" s="171"/>
-      <c r="N26" s="299" t="str">
+      <c r="N26" s="259" t="str">
         <f>CONCATENATE(M28,M29,M30,M31,M32,M33,M34,M35,M36,M37,M38,M39,M40)</f>
         <v/>
       </c>
@@ -6796,7 +6753,7 @@
       <c r="R26" s="131"/>
       <c r="S26" s="131"/>
     </row>
-    <row r="27" spans="2:19" s="70" customFormat="1" ht="22.9" customHeight="1" thickBot="1">
+    <row r="27" spans="2:19" s="70" customFormat="1" ht="22.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="132" t="s">
         <v>17</v>
       </c>
@@ -6812,7 +6769,7 @@
       <c r="F27" s="180" t="s">
         <v>2</v>
       </c>
-      <c r="G27" s="256"/>
+      <c r="G27" s="292"/>
       <c r="H27" s="103" t="s">
         <v>0</v>
       </c>
@@ -6823,16 +6780,16 @@
         <v>2</v>
       </c>
       <c r="K27" s="106"/>
-      <c r="L27" s="300"/>
+      <c r="L27" s="260"/>
       <c r="M27" s="171"/>
-      <c r="N27" s="300"/>
+      <c r="N27" s="260"/>
       <c r="O27" s="175"/>
       <c r="P27" s="106"/>
       <c r="Q27" s="106"/>
       <c r="R27" s="106"/>
       <c r="S27" s="106"/>
     </row>
-    <row r="28" spans="2:19" s="11" customFormat="1" ht="25.5" customHeight="1">
+    <row r="28" spans="2:19" s="11" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="134">
         <v>12</v>
       </c>
@@ -6845,7 +6802,7 @@
         <f t="shared" ref="F28:F39" si="2">IFERROR(D28/E28,)</f>
         <v>0</v>
       </c>
-      <c r="G28" s="256"/>
+      <c r="G28" s="292"/>
       <c r="H28" s="108" t="s">
         <v>46</v>
       </c>
@@ -6855,16 +6812,16 @@
         <f>IF(D28&gt;E28,"*Numerator for "&amp;C28&amp;" Cannot be more than Denominator"&amp;CHAR(10),"")</f>
         <v/>
       </c>
-      <c r="L28" s="300"/>
+      <c r="L28" s="260"/>
       <c r="M28" s="171"/>
-      <c r="N28" s="300"/>
+      <c r="N28" s="260"/>
       <c r="O28" s="175"/>
       <c r="P28" s="136"/>
       <c r="Q28" s="136"/>
       <c r="R28" s="136"/>
       <c r="S28" s="136"/>
     </row>
-    <row r="29" spans="2:19" s="11" customFormat="1" ht="25.5" customHeight="1">
+    <row r="29" spans="2:19" s="11" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="107">
         <v>13</v>
       </c>
@@ -6880,7 +6837,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G29" s="256"/>
+      <c r="G29" s="292"/>
       <c r="H29" s="108" t="s">
         <v>120</v>
       </c>
@@ -6892,16 +6849,16 @@
         <f t="shared" ref="K29:K32" si="3">IF(D29&gt;E29,"*Numerator for "&amp;C29&amp;" Cannot be more than Denominator"&amp;CHAR(10),"")</f>
         <v/>
       </c>
-      <c r="L29" s="300"/>
+      <c r="L29" s="260"/>
       <c r="M29" s="171"/>
-      <c r="N29" s="300"/>
+      <c r="N29" s="260"/>
       <c r="O29" s="175"/>
       <c r="P29" s="136"/>
       <c r="Q29" s="136"/>
       <c r="R29" s="136"/>
       <c r="S29" s="136"/>
     </row>
-    <row r="30" spans="2:19" s="11" customFormat="1" ht="25.5" customHeight="1">
+    <row r="30" spans="2:19" s="11" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="107">
         <v>14</v>
       </c>
@@ -6917,7 +6874,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G30" s="256"/>
+      <c r="G30" s="292"/>
       <c r="H30" s="108"/>
       <c r="I30" s="135" t="s">
         <v>120</v>
@@ -6927,16 +6884,16 @@
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="L30" s="300"/>
+      <c r="L30" s="260"/>
       <c r="M30" s="171"/>
-      <c r="N30" s="300"/>
+      <c r="N30" s="260"/>
       <c r="O30" s="175"/>
       <c r="P30" s="136"/>
       <c r="Q30" s="136"/>
       <c r="R30" s="136"/>
       <c r="S30" s="136"/>
     </row>
-    <row r="31" spans="2:19" s="11" customFormat="1" ht="25.5" customHeight="1">
+    <row r="31" spans="2:19" s="11" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="107">
         <v>15</v>
       </c>
@@ -6952,7 +6909,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G31" s="256"/>
+      <c r="G31" s="292"/>
       <c r="H31" s="137"/>
       <c r="I31" s="138"/>
       <c r="J31" s="124"/>
@@ -6960,16 +6917,16 @@
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="L31" s="300"/>
+      <c r="L31" s="260"/>
       <c r="M31" s="171"/>
-      <c r="N31" s="300"/>
+      <c r="N31" s="260"/>
       <c r="O31" s="175"/>
       <c r="P31" s="136"/>
       <c r="Q31" s="136"/>
       <c r="R31" s="136"/>
       <c r="S31" s="136"/>
     </row>
-    <row r="32" spans="2:19" s="12" customFormat="1" ht="25.5" customHeight="1" thickBot="1">
+    <row r="32" spans="2:19" s="12" customFormat="1" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="157">
         <v>16</v>
       </c>
@@ -6982,7 +6939,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G32" s="256"/>
+      <c r="G32" s="292"/>
       <c r="H32" s="108"/>
       <c r="I32" s="135" t="s">
         <v>47</v>
@@ -6992,19 +6949,19 @@
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="L32" s="300"/>
+      <c r="L32" s="260"/>
       <c r="M32" s="201" t="str">
         <f>IF(E32&gt;0,IF(D32/E32&lt;0.95,"*Linkage Rate amongest positive infants identified is below 95%"&amp;CHAR(10),""),"")</f>
         <v/>
       </c>
-      <c r="N32" s="300"/>
+      <c r="N32" s="260"/>
       <c r="O32" s="175"/>
       <c r="P32" s="139"/>
       <c r="Q32" s="139"/>
       <c r="R32" s="139"/>
       <c r="S32" s="139"/>
     </row>
-    <row r="33" spans="2:19" s="5" customFormat="1" ht="15" customHeight="1" thickBot="1">
+    <row r="33" spans="2:19" s="5" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B33" s="211">
         <v>17</v>
       </c>
@@ -7014,21 +6971,21 @@
       <c r="D33" s="213"/>
       <c r="E33" s="214"/>
       <c r="F33" s="215"/>
-      <c r="G33" s="256"/>
+      <c r="G33" s="292"/>
       <c r="H33" s="140"/>
       <c r="I33" s="141"/>
       <c r="J33" s="142"/>
       <c r="K33" s="131"/>
-      <c r="L33" s="300"/>
+      <c r="L33" s="260"/>
       <c r="M33" s="171"/>
-      <c r="N33" s="300"/>
+      <c r="N33" s="260"/>
       <c r="O33" s="176"/>
       <c r="P33" s="131"/>
       <c r="Q33" s="131"/>
       <c r="R33" s="131"/>
       <c r="S33" s="131"/>
     </row>
-    <row r="34" spans="2:19" s="6" customFormat="1" ht="25.5" customHeight="1">
+    <row r="34" spans="2:19" s="6" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="134">
         <v>17.100000000000001</v>
       </c>
@@ -7041,7 +6998,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G34" s="256"/>
+      <c r="G34" s="292"/>
       <c r="H34" s="143"/>
       <c r="I34" s="144" t="s">
         <v>77</v>
@@ -7051,16 +7008,16 @@
         <f>IF(SUM(D34:D39)&lt;&gt;E34,"*Sum of Numerator  17.1,17.2,17.3,17.4,17.5 and 17.6 should be equal to Denominator for 17.1","")</f>
         <v/>
       </c>
-      <c r="L34" s="300"/>
+      <c r="L34" s="260"/>
       <c r="M34" s="171"/>
-      <c r="N34" s="300"/>
+      <c r="N34" s="260"/>
       <c r="O34" s="173"/>
       <c r="P34" s="145"/>
       <c r="Q34" s="145"/>
       <c r="R34" s="145"/>
       <c r="S34" s="145"/>
     </row>
-    <row r="35" spans="2:19" s="6" customFormat="1" ht="25.5" customHeight="1">
+    <row r="35" spans="2:19" s="6" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="107">
         <v>17.2</v>
       </c>
@@ -7076,7 +7033,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G35" s="256"/>
+      <c r="G35" s="292"/>
       <c r="H35" s="146"/>
       <c r="I35" s="144" t="s">
         <v>77</v>
@@ -7086,16 +7043,16 @@
         <f>IF(D35&gt;E35,"*Numerator for "&amp;C35&amp;" Cannot be more than Denominator"&amp;CHAR(10),"")</f>
         <v/>
       </c>
-      <c r="L35" s="300"/>
+      <c r="L35" s="260"/>
       <c r="M35" s="171"/>
-      <c r="N35" s="300"/>
+      <c r="N35" s="260"/>
       <c r="O35" s="173"/>
       <c r="P35" s="145"/>
       <c r="Q35" s="145"/>
       <c r="R35" s="145"/>
       <c r="S35" s="145"/>
     </row>
-    <row r="36" spans="2:19" s="6" customFormat="1" ht="25.5" customHeight="1">
+    <row r="36" spans="2:19" s="6" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="107">
         <v>17.3</v>
       </c>
@@ -7114,7 +7071,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G36" s="256"/>
+      <c r="G36" s="292"/>
       <c r="H36" s="147" t="s">
         <v>47</v>
       </c>
@@ -7126,19 +7083,19 @@
         <f t="shared" ref="K36:K39" si="5">IF(D36&gt;E36,"*Numerator for "&amp;C36&amp;" Cannot be more than Denominator"&amp;CHAR(10),"")</f>
         <v/>
       </c>
-      <c r="L36" s="300"/>
+      <c r="L36" s="260"/>
       <c r="M36" s="201" t="str">
         <f>IF(E36&gt;0,IF(D36/E36&gt;0.05,"*EID Mother To Child Transmission rate is above 5%"&amp;CHAR(10),""),"")</f>
         <v/>
       </c>
-      <c r="N36" s="300"/>
+      <c r="N36" s="260"/>
       <c r="O36" s="173"/>
       <c r="P36" s="145"/>
       <c r="Q36" s="145"/>
       <c r="R36" s="145"/>
       <c r="S36" s="145"/>
     </row>
-    <row r="37" spans="2:19" s="6" customFormat="1" ht="25.5" customHeight="1">
+    <row r="37" spans="2:19" s="6" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="107">
         <v>17.399999999999999</v>
       </c>
@@ -7154,7 +7111,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G37" s="256"/>
+      <c r="G37" s="292"/>
       <c r="H37" s="108"/>
       <c r="I37" s="144" t="s">
         <v>77</v>
@@ -7164,16 +7121,16 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="L37" s="300"/>
+      <c r="L37" s="260"/>
       <c r="M37" s="171"/>
-      <c r="N37" s="300"/>
+      <c r="N37" s="260"/>
       <c r="O37" s="173"/>
       <c r="P37" s="145"/>
       <c r="Q37" s="145"/>
       <c r="R37" s="145"/>
       <c r="S37" s="145"/>
     </row>
-    <row r="38" spans="2:19" s="6" customFormat="1" ht="25.5" customHeight="1">
+    <row r="38" spans="2:19" s="6" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="107">
         <v>17.5</v>
       </c>
@@ -7189,7 +7146,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G38" s="256"/>
+      <c r="G38" s="292"/>
       <c r="H38" s="137"/>
       <c r="I38" s="144" t="s">
         <v>77</v>
@@ -7199,16 +7156,16 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="L38" s="300"/>
+      <c r="L38" s="260"/>
       <c r="M38" s="171"/>
-      <c r="N38" s="300"/>
+      <c r="N38" s="260"/>
       <c r="O38" s="173"/>
       <c r="P38" s="145"/>
       <c r="Q38" s="145"/>
       <c r="R38" s="145"/>
       <c r="S38" s="145"/>
     </row>
-    <row r="39" spans="2:19" s="6" customFormat="1" ht="25.5" customHeight="1" thickBot="1">
+    <row r="39" spans="2:19" s="6" customFormat="1" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B39" s="125">
         <v>17.600000000000001</v>
       </c>
@@ -7224,7 +7181,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G39" s="256"/>
+      <c r="G39" s="292"/>
       <c r="H39" s="126"/>
       <c r="I39" s="148" t="s">
         <v>77</v>
@@ -7234,27 +7191,27 @@
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="L39" s="301"/>
+      <c r="L39" s="261"/>
       <c r="M39" s="171"/>
-      <c r="N39" s="301"/>
+      <c r="N39" s="261"/>
       <c r="O39" s="173"/>
       <c r="P39" s="145"/>
       <c r="Q39" s="145"/>
       <c r="R39" s="145"/>
       <c r="S39" s="145"/>
     </row>
-    <row r="40" spans="2:19" s="8" customFormat="1" ht="15.75" customHeight="1">
-      <c r="B40" s="265" t="s">
+    <row r="40" spans="2:19" s="8" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="301" t="s">
         <v>79</v>
       </c>
-      <c r="C40" s="265"/>
-      <c r="D40" s="265"/>
-      <c r="E40" s="265"/>
-      <c r="F40" s="265"/>
-      <c r="G40" s="256"/>
-      <c r="H40" s="298"/>
-      <c r="I40" s="298"/>
-      <c r="J40" s="298"/>
+      <c r="C40" s="301"/>
+      <c r="D40" s="301"/>
+      <c r="E40" s="301"/>
+      <c r="F40" s="301"/>
+      <c r="G40" s="292"/>
+      <c r="H40" s="258"/>
+      <c r="I40" s="258"/>
+      <c r="J40" s="258"/>
       <c r="K40" s="149"/>
       <c r="L40" s="200"/>
       <c r="M40" s="171"/>
@@ -7266,20 +7223,8 @@
       <c r="S40" s="149"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="CnaItBN7QcJPUClG0sKbANpCkzo+GM8MGgPC8VfNZdywN+aHNeO+gOgYXMkH5BLRZN9Zgu70uwZ+6AuGpGP7sg==" saltValue="2PFSW0XVRtfQlmBmQ1v9mA==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="9WIGABGZM53eVaJNuSXz7Y7BjWjgxxLqL3EiPOJQ6O2IBwMiIUCcwrRgzWKjKRwdhtaIO9ArmYwxRFv25FSmHA==" saltValue="iE63twoK1TxISZ7/Y4fiXQ==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <mergeCells count="19">
-    <mergeCell ref="N8:N23"/>
-    <mergeCell ref="L8:L23"/>
-    <mergeCell ref="H26:J26"/>
-    <mergeCell ref="H40:J40"/>
-    <mergeCell ref="L26:L39"/>
-    <mergeCell ref="N26:N39"/>
-    <mergeCell ref="K1:O1"/>
-    <mergeCell ref="D5:F5"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="B2:S2"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="H3:J5"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="H6:J6"/>
@@ -7287,6 +7232,18 @@
     <mergeCell ref="B24:F25"/>
     <mergeCell ref="H24:J25"/>
     <mergeCell ref="B40:F40"/>
+    <mergeCell ref="K1:O1"/>
+    <mergeCell ref="D5:F5"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B2:S2"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="H3:J5"/>
+    <mergeCell ref="N8:N23"/>
+    <mergeCell ref="L8:L23"/>
+    <mergeCell ref="H26:J26"/>
+    <mergeCell ref="H40:J40"/>
+    <mergeCell ref="L26:L39"/>
+    <mergeCell ref="N26:N39"/>
   </mergeCells>
   <conditionalFormatting sqref="E9">
     <cfRule type="cellIs" dxfId="59" priority="100" operator="equal">

</xml_diff>